<commit_message>
Reescritura parcial de user stories del doc
Reescritura parcial de user stories del doc en función a lo observado en el USM.
</commit_message>
<xml_diff>
--- a/UserStories.xlsx
+++ b/UserStories.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>User Story</t>
   </si>
@@ -36,6 +36,63 @@
   </si>
   <si>
     <t>Criterios de Aceptación</t>
+  </si>
+  <si>
+    <t>Como ciudadano quiero poder registrarme para que retiren los elementos reciclables.</t>
+  </si>
+  <si>
+    <t>1) Debe pedir datos personales, horarios de retiro, y volúmen de los elementos reciclables.
+2) Debe permitir el ingreso opcional de una foto.
+3) Debe verificar que los datos ingresados sean verídicos.</t>
+  </si>
+  <si>
+    <t>Como cooperativa quiero poder asignar permisos especiales a mis empleados para que tengan acceso a información privada de la empresa.</t>
+  </si>
+  <si>
+    <t>1) Debe ser un proceso realizado por un superior.
+2) Debe identificarse mediante nombre de usuario y contraseña.</t>
+  </si>
+  <si>
+    <t>1) Designar usuario con permisos.
+2) Solicitar datos de usuario.
+3) Definir permisos.</t>
+  </si>
+  <si>
+    <t>Como cooperativa quiero atender las solicitudes de recolección para denegar aquellas que no cumplen ciertos requisitos.</t>
+  </si>
+  <si>
+    <t>1) Se deben denegar las solicitudes a una distancia mayor a 6 km del centro de acopio.
+2) Se debe avisar por mail el rechazo de la solicitud al ciudadano que hizo el pedido correspondiente.</t>
+  </si>
+  <si>
+    <t>1) Procesar las solicitudes.
+2) Da una respuesta por correo.</t>
+  </si>
+  <si>
+    <t>Como cooperativa quiero mostrar los materiales aceptados por el centro de acopio para informar a los interesados en aportar.</t>
+  </si>
+  <si>
+    <t>Como cooperativa quiero poder modificar los materiales aceptados que se muestran en la página para adaptarlo a la situación actual del centro de acopio.</t>
+  </si>
+  <si>
+    <t>1) Dicha modificación solo debe poder realizarla un usuario con permisos especiales.</t>
+  </si>
+  <si>
+    <t>1) Debe poder mostrarse una cantidad considerable, de manera tal que no sea una limitación.
+2) Debe ser flexible en la información que cuenta, opcionalmente con fotos.</t>
+  </si>
+  <si>
+    <t>1) Pedir datos.
+2) Verificar datos.</t>
+  </si>
+  <si>
+    <t>1) Verificar que el usuario tenga los permisos adecuados.
+2) Definir modificaciones en el catálogo.
+3) Actualizar la página.</t>
+  </si>
+  <si>
+    <t>1) Solicitar materiales e información.
+2) Incorporar al catálogo.</t>
   </si>
 </sst>
 </file>
@@ -483,7 +540,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.5703125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="79.140625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="73.42578125" style="11" customWidth="1"/>
     <col min="3" max="3" width="62.7109375" style="11" customWidth="1"/>
     <col min="4" max="4" width="36.140625" style="10" customWidth="1"/>
     <col min="5" max="16384" width="11.42578125" style="1"/>
@@ -503,45 +560,75 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="14"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="14"/>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="14"/>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="14"/>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="14"/>
+      <c r="B6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">

</xml_diff>